<commit_message>
Style earlier papers disclosure
</commit_message>
<xml_diff>
--- a/papers/Apaperinfo_to2020.xlsx
+++ b/papers/Apaperinfo_to2020.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="820" yWindow="680" windowWidth="27040" windowHeight="17560" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="27400" yWindow="620" windowWidth="26160" windowHeight="16940" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$G$50</definedName>
+  </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -69,14 +70,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,6 +445,7 @@
   <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
+    <col width="65.6640625" customWidth="1" min="1" max="1"/>
     <col width="62.33203125" customWidth="1" min="6" max="6"/>
     <col width="38.33203125" customWidth="1" min="7" max="7"/>
   </cols>
@@ -504,15 +505,15 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
+          <t>https://doi.org/10.1186/s13059-019-1824-y</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>43794</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Co-corresponding Author</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -537,10 +538,10 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
+          <t>https://doi.org/10.1073/pnas.1604558113</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>42598</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -570,19 +571,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
+          <t>https://doi.org/10.1093/bioinformatics/btx513</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>43084</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Joint Corresponding Author</t>
         </is>
       </c>
       <c r="G4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -603,10 +604,10 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
+          <t>https://doi.org/10.1038/nrclinonc.2018.30</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>43221</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -636,10 +637,10 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n">
+          <t>https://doi.org/10.1002/ijc.31014</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>43160</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -669,19 +670,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
+          <t>https://doi.org/10.2217/epi-2016-0153</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>42856</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>First Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -702,19 +703,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
+          <t>https://doi.org/10.1093/bioinformatics/btx622</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
         <v>43132</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Joint Corresponding Author</t>
         </is>
       </c>
       <c r="G8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -735,19 +736,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
+          <t>https://doi.org/10.2217/epi-2015-0017</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
         <v>42491</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -768,10 +769,10 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
+          <t>https://doi.org/10.1038/s41467-020-18618-y</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>44096</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -801,19 +802,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
+          <t>https://doi.org/10.1038/nrg.2017.86</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>43160</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>First Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -834,10 +835,10 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
+          <t>https://doi.org/10.1093/ije/dyz190</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
         <v>43739</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -867,15 +868,15 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
+          <t>https://doi.org/10.1186/s13073-020-00752-3</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>44006</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G13" t="b">
@@ -900,10 +901,10 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
+          <t>https://doi.org/10.1093/bioinformatics/btz456</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>43770</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -933,15 +934,15 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
+          <t>https://doi.org/10.1186/s13059-020-02126-9</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>44078</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G15" t="b">
@@ -966,19 +967,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
+          <t>https://doi.org/10.1093/bioinformatics/btz073</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>43723</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -999,10 +1000,10 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
+          <t>https://doi.org/10.1038/s41592-018-0213-x</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>43435</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1032,15 +1033,15 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
+          <t>https://doi.org/10.1186/s13059-018-1455-8</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
         <v>43259</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G18" t="b">
@@ -1065,19 +1066,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
+          <t>https://doi.org/10.1038/nmeth.4187</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>42794</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1098,10 +1099,10 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
+          <t>https://doi.org/10.1093/nar/gky882</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>43475</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1131,15 +1132,15 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
+          <t>https://doi.org/10.1093/nar/gkw1079</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>42739</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Joint Corresponding Author</t>
         </is>
       </c>
       <c r="G21" t="b">
@@ -1164,19 +1165,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n">
+          <t>https://doi.org/10.1038/s42003-019-0554-8</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
         <v>43686</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1197,19 +1198,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="n">
+          <t>https://doi.org/10.1038/ncomms15599</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>42887</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>First Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1230,19 +1231,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="n">
+          <t>https://doi.org/10.1038/s41525-020-00151-y</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
         <v>44111</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>First Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1263,15 +1264,15 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="n">
+          <t>https://doi.org/10.1038/s41563-018-0241-z</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>43586</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G25" t="b">
@@ -1296,10 +1297,10 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="n">
+          <t>https://doi.org/10.1016/j.celrep.2016.10.059</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>42689</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -1329,15 +1330,15 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n">
+          <t>https://doi.org/10.1186/s13059-016-1064-3</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>42646</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G27" t="b">
@@ -1362,19 +1363,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n">
+          <t>https://doi.org/10.18632/aging.101666</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
         <v>43431</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1395,19 +1396,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n">
+          <t>https://doi.org/10.1093/bioinformatics/btz833</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
         <v>43778</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1428,10 +1429,10 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n">
+          <t>https://doi.org/10.1007/978-1-4939-9057-3_9</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
         <v>43466</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -1461,10 +1462,10 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="n">
+          <t>https://doi.org/10.1038/ncomms13555</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
         <v>42703</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -1494,10 +1495,10 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="n">
+          <t>https://doi.org/10.1093/bib/bbx097</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
         <v>43483</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -1527,19 +1528,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="n">
+          <t>https://doi.org/10.1038/ncomms10478</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
         <v>42398</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>First Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -1560,10 +1561,10 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="n">
+          <t>https://doi.org/10.1093/nar/gkw1100</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>42760</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -1593,19 +1594,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="n">
+          <t>https://doi.org/10.2217/epi-2018-0037</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
         <v>43282</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1626,15 +1627,15 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="n">
+          <t>https://doi.org/10.1186/s12859-016-1056-z</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
         <v>42482</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G36" t="b">
@@ -1659,15 +1660,15 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="n">
+          <t>https://doi.org/10.1186/s13073-016-0342-8</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
         <v>42607</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G37" t="b">
@@ -1692,10 +1693,10 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="n">
+          <t>https://doi.org/10.1093/nar/gkw802</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
         <v>42719</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -1725,19 +1726,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="n">
+          <t>https://doi.org/10.1186/s13072-016-0058-4</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
         <v>42437</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -1758,19 +1759,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="n">
+          <t>https://doi.org/10.18632/aging.101533</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
         <v>43333</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>First Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -1791,19 +1792,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="n">
+          <t>https://doi.org/10.1093/bib/bby093</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
         <v>43847</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Joint Corresponding Author</t>
         </is>
       </c>
       <c r="G41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1824,10 +1825,10 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="n">
+          <t>https://doi.org/10.1186/s13073-017-0500-7</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
         <v>43091</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -1857,10 +1858,10 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n">
+          <t>https://doi.org/10.1093/hmg/ddy036</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
         <v>43191</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -1890,10 +1891,10 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="n">
+          <t>https://doi.org/10.1007/978-1-0716-0301-7_6</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
         <v>43831</v>
       </c>
       <c r="F44" t="inlineStr">
@@ -1923,15 +1924,15 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="n">
+          <t>https://doi.org/10.1186/s12859-017-1511-5</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
         <v>42779</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Corresponding Author</t>
+          <t>Main and Corresponding Author</t>
         </is>
       </c>
       <c r="G45" t="b">
@@ -1956,10 +1957,10 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="n">
+          <t>https://doi.org/10.1016/j.ebiom.2018.04.025</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
         <v>43221</v>
       </c>
       <c r="F46" t="inlineStr">
@@ -1989,19 +1990,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="n">
+          <t>https://doi.org/10.1093/cvr/cvx050</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n">
         <v>42856</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Co-author</t>
+          <t>Corresponding Author</t>
         </is>
       </c>
       <c r="G47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -2022,10 +2023,10 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="n">
+          <t>https://doi.org/10.1186/s13059-017-1366-0</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
         <v>43089</v>
       </c>
       <c r="F48" t="inlineStr">
@@ -2055,10 +2056,10 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="n">
+          <t>https://doi.org/10.1186/s13148-016-0231-4</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
         <v>42522</v>
       </c>
       <c r="F49" t="inlineStr">
@@ -2088,10 +2089,10 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://doi.org/10</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="n">
+          <t>https://doi.org/10.1097/igc.0000000000000739</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
         <v>42523</v>
       </c>
       <c r="F50" t="inlineStr">
@@ -2104,6 +2105,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>